<commit_message>
C13: run test case
</commit_message>
<xml_diff>
--- a/examples/config.xlsx
+++ b/examples/config.xlsx
@@ -1315,7 +1315,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Simulation type (LP or MILP)</t>
+          <t>Simulation type</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1332,7 +1332,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Solver time limit (seconds)</t>
+          <t>Solver time limit (s)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1379,7 +1379,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Edge elements for linearization</t>
+          <t>Edge elements</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1388,13 +1388,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Slack variable cost</t>
+          <t>Slack cost</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="10">
@@ -1495,13 +1495,13 @@
         </is>
       </c>
       <c r="D15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Temperature cyclic constraint</t>
+          <t>Temperature cyclic</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1516,7 +1516,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bypass cyclic constraint</t>
+          <t>Bypass cyclic</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1531,7 +1531,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Turbine cyclic constraint</t>
+          <t>Turbine cyclic</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1540,13 +1540,13 @@
         </is>
       </c>
       <c r="D18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Total release cyclic constraint</t>
+          <t>Total cyclic</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1555,13 +1555,13 @@
         </is>
       </c>
       <c r="D19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gauge cyclic constraint</t>
+          <t>Gauge cyclic</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1570,13 +1570,13 @@
         </is>
       </c>
       <c r="D20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Operating range constraint</t>
+          <t>Operating range</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1591,7 +1591,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Rough zone constraint</t>
+          <t>Rough zone</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1606,7 +1606,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pattern repeat mode</t>
+          <t>Pattern repeat</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1691,7 +1691,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Plant to node mapping</t>
+          <t>Plant to node</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1708,7 +1708,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Source nodes</t>
+          <t>Sources</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1725,7 +1725,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sink nodes</t>
+          <t>Sinks</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1756,31 +1756,31 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>240000</v>
+        <v>19835</v>
       </c>
       <c r="F31" t="n">
-        <v>240000</v>
+        <v>19835</v>
       </c>
       <c r="G31" t="n">
-        <v>240000</v>
+        <v>19835</v>
       </c>
       <c r="H31" t="n">
-        <v>240000</v>
+        <v>19835</v>
       </c>
       <c r="I31" t="n">
-        <v>240000</v>
+        <v>19835</v>
       </c>
       <c r="J31" t="n">
-        <v>240000</v>
+        <v>19835</v>
       </c>
       <c r="K31" t="n">
-        <v>240000</v>
+        <v>19835</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Total daily release (AF) - gauge</t>
+          <t>Total daily release - gauge</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1818,7 +1818,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Max daily flow change (CFS)</t>
+          <t>Max daily change (CFS)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1856,7 +1856,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Max daily flow change - gauge</t>
+          <t>Max daily change - gauge</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1894,7 +1894,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Water to power conversion (MW/CFS)</t>
+          <t>Water-to-power (MW/CFS)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1932,7 +1932,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Water to power conversion - gauge</t>
+          <t>Water-to-power - gauge</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1970,7 +1970,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Daily gauge temperature max (C)</t>
+          <t>Daily gauge temp max</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2008,7 +2008,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Daily gauge temperature max (C)</t>
+          <t>Daily gauge temp max</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2046,7 +2046,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Daily temperature delta</t>
+          <t>Daily temp delta</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2084,7 +2084,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Bypass ramp up max (CFS/hr)</t>
+          <t>Q_bp_ramp_up_max</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2104,7 +2104,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Bypass ramp up max (CFS/hr) - gauge</t>
+          <t>Q_bp_ramp_up_max - gauge</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2124,7 +2124,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Bypass ramp down max (CFS/hr)</t>
+          <t>Q_bp_ramp_down_max</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2144,7 +2144,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Bypass ramp down max (CFS/hr) - gauge</t>
+          <t>Q_bp_ramp_down_max - gauge</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2164,7 +2164,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Turbine ramp up max (CFS/hr)</t>
+          <t>Q_tur_ramp_up_max</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2184,7 +2184,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Turbine ramp up max (CFS/hr) - gauge</t>
+          <t>Q_tur_ramp_up_max - gauge</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2204,7 +2204,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Turbine ramp down max (CFS/hr)</t>
+          <t>Q_tur_ramp_down_max</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2224,7 +2224,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Turbine ramp down max (CFS/hr) - gauge</t>
+          <t>Q_tur_ramp_down_max - gauge</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2244,7 +2244,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Total ramp up max (CFS/hr)</t>
+          <t>Q_tot_ramp_up_max</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Total ramp up max (CFS/hr) - gauge</t>
+          <t>Q_tot_ramp_up_max - gauge</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2284,7 +2284,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Total ramp down max (CFS/hr)</t>
+          <t>Q_tot_ramp_down_max</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2304,7 +2304,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Total ramp down max (CFS/hr) - gauge</t>
+          <t>Q_tot_ramp_down_max - gauge</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2324,7 +2324,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Gauge ramp up max (CFS/hr)</t>
+          <t>Q_gg_ramp_up_max</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2344,7 +2344,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Gauge ramp up max (CFS/hr) - gauge</t>
+          <t>Q_gg_ramp_up_max - gauge</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2364,7 +2364,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Gauge ramp down max (CFS/hr)</t>
+          <t>Q_gg_ramp_down_max</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2384,7 +2384,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Gauge ramp down max (CFS/hr) - gauge</t>
+          <t>Q_gg_ramp_down_max - gauge</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2404,7 +2404,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Bypass ramp up cycles per day</t>
+          <t>bp_ramp_up_cyc</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Bypass ramp up cycles per day - gauge</t>
+          <t>bp_ramp_up_cyc - gauge</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2444,7 +2444,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Bypass ramp down cycles per day</t>
+          <t>bp_ramp_down_cyc</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2464,7 +2464,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Bypass ramp down cycles per day - gauge</t>
+          <t>bp_ramp_down_cyc - gauge</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2484,7 +2484,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Bypass total ramp cycles per day</t>
+          <t>bp_ramp_tot_cyc</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2498,13 +2498,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Bypass total ramp cycles per day - gauge</t>
+          <t>bp_ramp_tot_cyc - gauge</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2524,7 +2524,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Cost bypass ramp up ($/CFS)</t>
+          <t>C_bp_ramp_up</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2544,7 +2544,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Cost bypass ramp up ($/CFS) - gauge</t>
+          <t>C_bp_ramp_up - gauge</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2564,7 +2564,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Cost bypass ramp down ($/CFS)</t>
+          <t>C_bp_ramp_down</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2584,7 +2584,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cost bypass ramp down ($/CFS) - gauge</t>
+          <t>C_bp_ramp_down - gauge</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2604,7 +2604,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Cost turbine ramp up ($/CFS)</t>
+          <t>C_tur_ramp_up</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2624,7 +2624,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Cost turbine ramp up ($/CFS) - gauge</t>
+          <t>C_tur_ramp_up - gauge</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2644,7 +2644,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Cost turbine ramp down ($/CFS)</t>
+          <t>C_tur_ramp_down</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2664,7 +2664,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Cost turbine ramp down ($/CFS) - gauge</t>
+          <t>C_tur_ramp_down - gauge</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2684,7 +2684,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cost total ramp up ($/CFS)</t>
+          <t>C_tot_ramp_up</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2698,13 +2698,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Cost total ramp up ($/CFS) - gauge</t>
+          <t>C_tot_ramp_up - gauge</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2724,7 +2724,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Cost total ramp down ($/CFS)</t>
+          <t>C_tot_ramp_down</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2738,13 +2738,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Cost total ramp down ($/CFS) - gauge</t>
+          <t>C_tot_ramp_down - gauge</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2764,7 +2764,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Cost gauge ramp up ($/CFS)</t>
+          <t>C_gg_ramp_up</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2778,13 +2778,13 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Cost gauge ramp up ($/CFS) - gauge</t>
+          <t>C_gg_ramp_up - gauge</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2804,7 +2804,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Cost gauge ramp down ($/CFS)</t>
+          <t>C_gg_ramp_down</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2818,13 +2818,13 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Cost gauge ramp down ($/CFS) - gauge</t>
+          <t>C_gg_ramp_down - gauge</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2844,7 +2844,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Bypass min flow (CFS)</t>
+          <t>Bypass min (CFS)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3365,7 +3365,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Bypass min flow - gauge</t>
+          <t>Bypass min - gauge</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3886,7 +3886,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Bypass max flow (CFS)</t>
+          <t>Bypass max (CFS)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4407,7 +4407,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Bypass max flow - gauge</t>
+          <t>Bypass max - gauge</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4928,7 +4928,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Turbine min flow (CFS)</t>
+          <t>Turbine min (CFS)</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -5449,7 +5449,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Turbine min flow - gauge</t>
+          <t>Turbine min - gauge</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -5970,7 +5970,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Turbine max flow (CFS)</t>
+          <t>Turbine max (CFS)</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -6491,7 +6491,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Turbine max flow - gauge</t>
+          <t>Turbine max - gauge</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -7012,7 +7012,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Total min flow (CFS)</t>
+          <t>Total min (CFS)</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -7533,7 +7533,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Total min flow - gauge</t>
+          <t>Total min - gauge</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -8054,7 +8054,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Total max flow (CFS)</t>
+          <t>Total max (CFS)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -8575,7 +8575,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Total max flow - gauge</t>
+          <t>Total max - gauge</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -9096,7 +9096,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Gauge min flow (CFS)</t>
+          <t>Gauge min (CFS)</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -9617,7 +9617,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Gauge min flow - gauge</t>
+          <t>Gauge min - gauge</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -10138,7 +10138,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Gauge max flow (CFS)</t>
+          <t>Gauge max (CFS)</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -10659,7 +10659,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Gauge max flow - gauge</t>
+          <t>Gauge max - gauge</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -11180,7 +11180,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Bypass temperature (C)</t>
+          <t>Bypass temp (C)</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -11701,7 +11701,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Bypass temperature - gauge</t>
+          <t>Bypass temp - gauge</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -12222,7 +12222,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Turbine temperature (C)</t>
+          <t>Turbine temp (C)</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -12236,514 +12236,514 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="S96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="T96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="U96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="W96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="X96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Y96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Z96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AA96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AB96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AC96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AD96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AE96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AF96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AG96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AH96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AI96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AJ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AK96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AL96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AM96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AN96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AO96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AP96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AQ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AR96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AS96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AT96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AU96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AV96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AW96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AX96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AY96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AZ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BA96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BB96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BC96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BD96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BE96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BF96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BG96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BH96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BI96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BJ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BK96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BL96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BM96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BN96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BO96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BP96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BQ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BR96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BS96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BT96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BU96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BV96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BW96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BX96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BY96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BZ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CA96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CB96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CC96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CD96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CE96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CF96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CG96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CH96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CI96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CJ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CK96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CL96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CM96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CN96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CO96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CP96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CQ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CR96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CS96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CT96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CU96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CV96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CW96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CX96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CY96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CZ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DA96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DB96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DC96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DD96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DE96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DF96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DG96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DH96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DI96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DJ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DK96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DL96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DM96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DN96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DO96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DP96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DQ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DR96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DS96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DT96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DU96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DV96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DW96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DX96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DY96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="DZ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EA96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EB96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EC96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="ED96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EE96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EF96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EG96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EH96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EI96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EJ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EK96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EL96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EM96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EN96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EO96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EP96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EQ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="ER96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="ES96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="ET96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EU96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EV96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EW96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EX96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EY96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EZ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FA96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FB96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FC96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FD96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FE96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FF96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FG96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FH96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FI96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FJ96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FK96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FL96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FM96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FN96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FO96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="FP96" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Turbine temperature - gauge</t>
+          <t>Turbine temp - gauge</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -13264,7 +13264,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Gauge hourly min temperature (C)</t>
+          <t>Gauge hourly min temp (C)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -13785,7 +13785,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Gauge hourly max temperature (C)</t>
+          <t>Gauge hourly max temp (C)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -13799,514 +13799,514 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="U99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="V99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="W99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="X99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Y99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Z99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AA99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AB99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AC99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AD99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AE99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AF99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AG99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AH99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AI99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AJ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AK99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AL99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AM99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AN99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AO99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AP99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AQ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AR99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AS99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AT99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AU99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AV99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AW99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AX99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AY99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AZ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BA99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BB99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BC99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BD99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BE99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BF99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BG99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BH99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BI99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BJ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BK99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BL99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BM99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BN99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BO99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BP99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BQ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BR99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BS99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BT99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BU99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BV99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BW99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BX99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BY99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BZ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CA99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CB99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CC99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CD99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CE99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CF99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CG99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CH99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CI99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CJ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CK99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CL99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CM99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CN99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CO99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CP99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CQ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CR99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CS99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CT99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CU99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CV99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CW99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CX99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CY99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="CZ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DA99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DB99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DC99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DD99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DE99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DF99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DG99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DH99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DI99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DJ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DK99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DL99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DM99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DN99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DO99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DP99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DQ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DR99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DS99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DT99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DU99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DV99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DW99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DX99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DY99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="DZ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EA99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EB99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EC99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="ED99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EE99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EF99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EG99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EH99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EI99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EJ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EK99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EL99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EM99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EN99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EO99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EP99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EQ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="ER99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="ES99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="ET99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EU99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EV99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EW99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EX99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EY99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="EZ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FA99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FB99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FC99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FD99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FE99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FF99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FG99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FH99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FI99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FJ99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FK99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FL99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FM99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FN99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FO99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="FP99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Hourly temperature delta (C)</t>
+          <t>Hourly temp delta (C)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -14827,7 +14827,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Power output min (MW)</t>
+          <t>Power min (MW)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -15348,7 +15348,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Power output min - gauge</t>
+          <t>Power min - gauge</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -15869,7 +15869,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Power output max (MW)</t>
+          <t>Power max (MW)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -15883,514 +15883,514 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="F103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="G103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="H103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="I103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="J103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="K103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="L103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="M103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="N103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="O103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="P103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="Q103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="R103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="S103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="T103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="U103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="V103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="W103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="X103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="Y103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="Z103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AA103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AB103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AC103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AD103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AE103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AF103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AG103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AH103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AI103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AJ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AK103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AL103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AM103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AN103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AO103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AP103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AQ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AR103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AS103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AT103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AU103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AV103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AW103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AX103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AY103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="AZ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BA103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BB103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BC103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BD103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BE103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BF103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BG103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BH103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BI103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BJ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BK103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BL103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BM103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BN103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BO103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BP103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BQ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BR103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BS103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BT103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BU103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BV103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BW103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BX103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BY103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="BZ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CA103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CB103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CC103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CD103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CE103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CF103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CG103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CH103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CI103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CJ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CK103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CL103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CM103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CN103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CO103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CP103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CQ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CR103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CS103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CT103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CU103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CV103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CW103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CX103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CY103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="CZ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DA103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DB103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DC103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DD103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DE103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DF103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DG103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DH103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DI103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DJ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DK103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DL103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DM103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DN103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DO103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DP103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DQ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DR103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DS103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DT103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DU103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DV103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DW103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DX103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DY103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="DZ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EA103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EB103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EC103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="ED103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EE103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EF103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EG103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EH103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EI103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EJ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EK103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EL103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EM103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EN103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EO103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EP103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EQ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="ER103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="ES103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="ET103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EU103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EV103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EW103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EX103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EY103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="EZ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FA103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FB103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FC103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FD103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FE103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FF103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FG103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FH103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FI103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FJ103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FK103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FL103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FM103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FN103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FO103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
       <c r="FP103" t="n">
-        <v>150</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Power output max - gauge</t>
+          <t>Power max - gauge</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -16911,7 +16911,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Bypass forced commit status</t>
+          <t>Bypass forced commit</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -17953,7 +17953,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Max flow between nodes (CFS)</t>
+          <t>Max flow i-j (CFS)</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -18474,7 +18474,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Min flow between nodes (CFS)</t>
+          <t>Min flow i-j (CFS)</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -18995,7 +18995,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Source hourly max temperature (C)</t>
+          <t>Source max temp (C)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -19516,7 +19516,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Source hourly min temperature (C)</t>
+          <t>Source min temp (C)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -20037,7 +20037,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Sink hourly max temperature (C)</t>
+          <t>Sink max temp (C)</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -20558,7 +20558,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Sink hourly min temperature (C)</t>
+          <t>Sink min temp (C)</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -21079,7 +21079,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Temperature ramp up delta (C)</t>
+          <t>Temp ramp up delta</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -21093,13 +21093,13 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Temperature ramp up delta - gauge</t>
+          <t>Temp ramp up delta - gauge</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -21113,13 +21113,13 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Temperature ramp down delta (C)</t>
+          <t>Temp ramp down delta</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -21133,13 +21133,13 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Temperature ramp down delta - gauge</t>
+          <t>Temp ramp down delta - gauge</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -21153,13 +21153,13 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Locational marginal price ($/MWh)</t>
+          <t>LMP ($/MWh)</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -22201,7 +22201,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Rough zone min flow (CFS)</t>
+          <t>Rough zone min (CFS)</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -22219,15 +22219,12 @@
       </c>
       <c r="F119" t="n">
         <v>4000</v>
-      </c>
-      <c r="G119" t="n">
-        <v>6800</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Rough zone max flow (CFS)</t>
+          <t>Rough zone max (CFS)</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -22245,9 +22242,6 @@
       </c>
       <c r="F120" t="n">
         <v>4800</v>
-      </c>
-      <c r="G120" t="n">
-        <v>7200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>